<commit_message>
Weekly update · 2026-05-18
</commit_message>
<xml_diff>
--- a/big_ideas_2026-05-15.xlsx
+++ b/big_ideas_2026-05-15.xlsx
@@ -10139,7 +10139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10207,44 +10207,24 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>WEEKLY_UPDATE</t>
+          <t>BASE_RUN</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Heavy commercialization week across bio and AI infrastructure. In bio: Isomorphic Labs closed a $2.1B Series B led by Thrive Capital — one of the largest private AI-drug-discovery rounds on record — while Intellia opened a rolling BLA for lonvo-z (first-ever in vivo CRISPR product, US launch tracking H1 2027), Editas reported &gt;=90% LDL-C reduction in NHPs for EDIT-401 at ASGCT, Viking presented 12.2% 13-week weight loss for oral VK2735 at ECO 2026, and Neuralink signaled a next-gen 'whole-brain' surgical robot. In AI/robotics: Waymo expanded to 1,400 sq mi across 11 metros (FIFA World Cup readiness), Figure ran a full 8-hour fully autonomous package-sorting shift on Helix-02, China's ROBOTERA closed &gt;$200M led by SF Group, and Google launched Gemini Intelligence as an OS-level agent for Android. Energy/quantum: CATL announced a 40 GWh sodium-ion expansion, BNEF confirmed energy storage entered the '100 GW era' in 2025, Ford launched a 20 GWh/yr LFP grid-storage subsidiary, IonQ shareholders approved the $1.8B SkyWater acquisition, and Google added Marvell as a third TPU partner targeting ~2M inference MPUs. Agent D flagged three adjacencies: Archer's UAE Restricted Type Certificate path (first eVTOL on this pathway), the EU AI Act omnibus simplification (and nudification ban), and an HKU ultra-stainless-steel claim that could cut seawater-electrolysis structural costs ~40x.</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>UPDATED_FACT</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>#11 Self-driving cars / robotaxis</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Waymo expands robotaxi coverage to 1,400 sq mi across 11 US cities</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>On May 13, 2026, Waymo announced a 20%+ expansion of service area to over 1,400 square miles across 11 US cities, rolling out from Miami to Austin, Atlanta, Houston and the SF Bay Area, timed to FIFA World Cup readiness.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>https://waymo.com/blog/shorts/growing-to-1400-sqm/ | https://electrek.co/2026/05/13/waymo-expands-coverage-1400-square-miles-11-cities/</t>
-        </is>
-      </c>
+          <t>Seeded 'voices' section with 16 curated thinkers across AI, bio, energy, space, and macro tech.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -10269,22 +10249,22 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>#12 Humanoid robotics</t>
+          <t>#11 Self-driving cars / robotaxis</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Figure Helix-02 runs full 8-hour autonomous package-sorting shift</t>
+          <t>Waymo expands robotaxi coverage to 1,400 sq mi across 11 US cities</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>On May 13, 2026, Figure AI demonstrated Helix-02-equipped humanoids sustaining a continuous 8-hour package-sorting shift at near-human throughput (~3 sec/package), claimed to be the first eight-hour fully autonomous humanoid factory shift.</t>
+          <t>On May 13, 2026, Waymo announced a 20%+ expansion of service area to over 1,400 square miles across 11 US cities, rolling out from Miami to Austin, Atlanta, Houston and the SF Bay Area, timed to FIFA World Cup readiness.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://interestingengineering.com/ai-robotics/figure-helix02-humanoid-robots-8-hour-shifts | https://www.techtimes.com/articles/316632/20260514/figure-ais-helix-02-robots-complete-full-8-hour-autonomous-shifts-humanoid-race-intensifies.htm</t>
+          <t>https://waymo.com/blog/shorts/growing-to-1400-sqm/ | https://electrek.co/2026/05/13/waymo-expands-coverage-1400-square-miles-11-cities/</t>
         </is>
       </c>
     </row>
@@ -10306,7 +10286,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>NEW_WATCH</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -10316,17 +10296,17 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>ROBOTERA closes &gt;$200M led by SF Group, HSG, IDG to scale humanoid fleet</t>
+          <t>Figure Helix-02 runs full 8-hour autonomous package-sorting shift</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>On May 8, 2026, Chinese humanoid maker ROBOTERA closed &gt;$200M (SF Group, HSG, IDG Capital, Hillhouse, Alibaba, Geely, Lenovo, etc.) after Q2 thousand-unit deliveries and 300%+ growth in logistics deployments.</t>
+          <t>On May 13, 2026, Figure AI demonstrated Helix-02-equipped humanoids sustaining a continuous 8-hour package-sorting shift at near-human throughput (~3 sec/package), claimed to be the first eight-hour fully autonomous humanoid factory shift.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/robotera-raises-over-usd-200-million-in-new-round-led-by-sf-group-hsg-and-idg-capital-302766752.html | https://theaiinsider.tech/2026/05/08/chinas-humanoid-robot-maker-robotera-raises-over-usd-200m-in-new-funding-round/</t>
+          <t>https://interestingengineering.com/ai-robotics/figure-helix02-humanoid-robots-8-hour-shifts | https://www.techtimes.com/articles/316632/20260514/figure-ais-helix-02-robots-complete-full-8-hour-autonomous-shifts-humanoid-race-intensifies.htm</t>
         </is>
       </c>
     </row>
@@ -10348,27 +10328,27 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
+          <t>NEW_WATCH</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>#01 Transformers / LLMs / coding agents</t>
+          <t>#12 Humanoid robotics</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Google launches Gemini Intelligence as an OS-level agentic layer on Android</t>
+          <t>ROBOTERA closes &gt;$200M led by SF Group, HSG, IDG to scale humanoid fleet</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>At the Android Show on May 12, 2026, Google unveiled Gemini Intelligence, an agentic layer that reads on-screen context and executes cross-app, multi-step tasks (shopping, forms, dictation, vibe-coded widgets) on Pixel and Galaxy devices starting summer 2026.</t>
+          <t>On May 8, 2026, Chinese humanoid maker ROBOTERA closed &gt;$200M (SF Group, HSG, IDG Capital, Hillhouse, Alibaba, Geely, Lenovo, etc.) after Q2 thousand-unit deliveries and 300%+ growth in logistics deployments.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://blog.google/security/android-gemini-intelligence-security-privacy/ | https://techcrunch.com/2026/05/12/google-brings-agentic-ai-and-vibe-coded-widgets-to-android/</t>
+          <t>https://www.prnewswire.com/news-releases/robotera-raises-over-usd-200-million-in-new-round-led-by-sf-group-hsg-and-idg-capital-302766752.html | https://theaiinsider.tech/2026/05/08/chinas-humanoid-robot-maker-robotera-raises-over-usd-200m-in-new-funding-round/</t>
         </is>
       </c>
     </row>
@@ -10390,27 +10370,27 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>NEW_SUB_IDEA</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>#04 AlphaFold + computational protein design</t>
+          <t>#01 Transformers / LLMs / coding agents</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Isomorphic Labs raises $2.1B Series B for AI drug-design engine</t>
+          <t>Google launches Gemini Intelligence as an OS-level agentic layer on Android</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>On May 12, 2026, Alphabet-backed Isomorphic Labs announced a $2.1B Series B led by Thrive Capital (with Alphabet, GV, MGX, Temasek, CapitalG, UK Sovereign AI Fund) to scale IsoDDE and push its in-house pipeline toward the clinic.</t>
+          <t>At the Android Show on May 12, 2026, Google unveiled Gemini Intelligence, an agentic layer that reads on-screen context and executes cross-app, multi-step tasks (shopping, forms, dictation, vibe-coded widgets) on Pixel and Galaxy devices starting summer 2026.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>https://www.isomorphiclabs.com/articles/isomorphic-labs-announces-series-b-investment-round | https://www.prnewswire.com/news-releases/isomorphic-labs-secures-2-1-billion-funding-to-scale-its-ai-drug-design-engine-302769674.html</t>
+          <t>https://blog.google/security/android-gemini-intelligence-security-privacy/ | https://techcrunch.com/2026/05/12/google-brings-agentic-ai-and-vibe-coded-widgets-to-android/</t>
         </is>
       </c>
     </row>
@@ -10432,27 +10412,27 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>#07 CRISPR therapies (Casgevy + base/prime editing)</t>
+          <t>#04 AlphaFold + computational protein design</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Intellia initiates rolling BLA for lonvo-z after Phase 3 HAELO data</t>
+          <t>Isomorphic Labs raises $2.1B Series B for AI drug-design engine</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>In Q1 2026 results released May 11, Intellia confirmed Phase 3 HAELO topline for in vivo CRISPR therapy lonvo-z showed 87% reduction in HAE attacks vs placebo over six months with 62% attack-free/therapy-free patients; rolling BLA initiated with submission completion targeted H2 2026 and potential US launch H1 2027.</t>
+          <t>On May 12, 2026, Alphabet-backed Isomorphic Labs announced a $2.1B Series B led by Thrive Capital (with Alphabet, GV, MGX, Temasek, CapitalG, UK Sovereign AI Fund) to scale IsoDDE and push its in-house pipeline toward the clinic.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/11/3291773/0/en/Intellia-Therapeutics-Announces-First-Quarter-2026-Financial-Results-and-Business-Updates.html | https://ir.intelliatx.com/news-releases/news-release-details/intellia-therapeutics-announces-first-quarter-2026-financial</t>
+          <t>https://www.isomorphiclabs.com/articles/isomorphic-labs-announces-series-b-investment-round | https://www.prnewswire.com/news-releases/isomorphic-labs-secures-2-1-billion-funding-to-scale-its-ai-drug-design-engine-302769674.html</t>
         </is>
       </c>
     </row>
@@ -10474,7 +10454,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>NEW_WATCH</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -10484,17 +10464,17 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Editas EDIT-401 hits &gt;=90% LDL-C reduction in NHPs at ASGCT 2026</t>
+          <t>Intellia initiates rolling BLA for lonvo-z after Phase 3 HAELO data</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>On May 14, 2026, Editas reported at ASGCT 2026 that a single dose of in vivo gene-editing candidate EDIT-401 achieved &gt;=90% mean LDL-C reduction across dose groups in non-human primates via LDLR upregulation; first-in-human in HeFH planned later this year with early human PoC by year-end.</t>
+          <t>In Q1 2026 results released May 11, Intellia confirmed Phase 3 HAELO topline for in vivo CRISPR therapy lonvo-z showed 87% reduction in HAE attacks vs placebo over six months with 62% attack-free/therapy-free patients; rolling BLA initiated with submission completion targeted H2 2026 and potential US launch H1 2027.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/14/3294685/0/en/editas-medicine-reports-new-preclinical-data-demonstrating-progress-of-edit-401-as-potential-treatment-for-hyperlipidemia-at-the-american-society-of-gene-and-cell-therapy-2026-annu.html | https://ir.editasmedicine.com/news-releases/news-release-details/editas-medicine-nominates-edit-401-ldlr-targeted-medicine-lead</t>
+          <t>https://www.globenewswire.com/news-release/2026/05/11/3291773/0/en/Intellia-Therapeutics-Announces-First-Quarter-2026-Financial-Results-and-Business-Updates.html | https://ir.intelliatx.com/news-releases/news-release-details/intellia-therapeutics-announces-first-quarter-2026-financial</t>
         </is>
       </c>
     </row>
@@ -10516,27 +10496,27 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_WATCH</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>#06 GLP-1 agonists</t>
+          <t>#07 CRISPR therapies (Casgevy + base/prime editing)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Viking VK2735 oral hits 12.2% weight loss at 13 weeks (ECO 2026)</t>
+          <t>Editas EDIT-401 hits &gt;=90% LDL-C reduction in NHPs at ASGCT 2026</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>At the European Congress on Obesity in Istanbul on May 12, 2026, Viking presented Phase 2 VENTURE-Oral 13-week data showing oral VK2735 delivered up to 12.2% mean weight loss with no plateau, 97% of treated patients hitting &gt;=5% weight loss vs 10% placebo; subcutaneous Phase 3 VANQUISH-1 trial design also presented.</t>
+          <t>On May 14, 2026, Editas reported at ASGCT 2026 that a single dose of in vivo gene-editing candidate EDIT-401 achieved &gt;=90% mean LDL-C reduction across dose groups in non-human primates via LDLR upregulation; first-in-human in HeFH planned later this year with early human PoC by year-end.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/viking-therapeutics-presents-data-from-its-13-week-phase-2-venture-oral-dosing-trial-of-vk2735-at-european-congress-on-obesity-eco-2026-302768959.html</t>
+          <t>https://www.globenewswire.com/news-release/2026/05/14/3294685/0/en/editas-medicine-reports-new-preclinical-data-demonstrating-progress-of-edit-401-as-potential-treatment-for-hyperlipidemia-at-the-american-society-of-gene-and-cell-therapy-2026-annu.html | https://ir.editasmedicine.com/news-releases/news-release-details/editas-medicine-nominates-edit-401-ldlr-targeted-medicine-lead</t>
         </is>
       </c>
     </row>
@@ -10558,27 +10538,27 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>#14 Brain-computer interfaces</t>
+          <t>#06 GLP-1 agonists</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Neuralink unveils next-gen surgical robot for whole-brain access</t>
+          <t>Viking VK2735 oral hits 12.2% weight loss at 13 weeks (ECO 2026)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>On May 7-8, 2026, Elon Musk announced Neuralink is developing a next-generation surgical robot designed to implant electrode threads in any region of the brain with high precision, signaling a push beyond motor cortex into Parkinson's, epilepsy, and sensory disorders and toward high-volume implant production in 2026.</t>
+          <t>At the European Congress on Obesity in Istanbul on May 12, 2026, Viking presented Phase 2 VENTURE-Oral 13-week data showing oral VK2735 delivered up to 12.2% mean weight loss with no plateau, 97% of treated patients hitting &gt;=5% weight loss vs 10% placebo; subcutaneous Phase 3 VANQUISH-1 trial design also presented.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>https://www.foxnews.com/health/elon-musk-shares-plan-mass-produce-brain-implants-paralysis-neurological-disease | https://yourstory.com/2026/05/neuralink-surgical-robot-brain-interface-2026</t>
+          <t>https://www.prnewswire.com/news-releases/viking-therapeutics-presents-data-from-its-13-week-phase-2-venture-oral-dosing-trial-of-vk2735-at-european-congress-on-obesity-eco-2026-302768959.html</t>
         </is>
       </c>
     </row>
@@ -10600,27 +10580,27 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>#07 CRISPR therapies (Casgevy + base/prime editing)</t>
+          <t>#14 Brain-computer interfaces</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Casgevy hits $43M Q1 revenue with 500+ patients initiated</t>
+          <t>Neuralink unveils next-gen surgical robot for whole-brain access</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>CRISPR Therapeutics Q1 2026 results (released early May) showed Casgevy revenue of $43.0M with over 500 patients initiated globally, marking continued ramp of the first commercial CRISPR therapy; company holds $2.44B cash with multiple in vivo CRISPR INDs (CTX310, CTX460, CTX340) advancing.</t>
+          <t>On May 7-8, 2026, Elon Musk announced Neuralink is developing a next-generation surgical robot designed to implant electrode threads in any region of the brain with high precision, signaling a push beyond motor cortex into Parkinson's, epilepsy, and sensory disorders and toward high-volume implant production in 2026.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.stocktitan.net/news/CRSP/crispr-therapeutics-provides-business-update-and-reports-first-sdrpmbu7dwil.html | https://ir.crisprtx.com/</t>
+          <t>https://www.foxnews.com/health/elon-musk-shares-plan-mass-produce-brain-implants-paralysis-neurological-disease | https://yourstory.com/2026/05/neuralink-surgical-robot-brain-interface-2026</t>
         </is>
       </c>
     </row>
@@ -10647,22 +10627,22 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>#08 Quantum error correction (logical qubits below threshold)</t>
+          <t>#07 CRISPR therapies (Casgevy + base/prime editing)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>IonQ-SkyWater $1.8B merger clears shareholder vote</t>
+          <t>Casgevy hits $43M Q1 revenue with 500+ patients initiated</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>SkyWater Technology stockholders approved IonQ's ~$1.8B cash-and-stock acquisition at a May 8, 2026 special meeting (32.6M for, 405K against). Deal makes IonQ the only vertically integrated full-stack quantum platform with an in-house US semiconductor fab; closing expected Q2-Q3 2026 pending regulatory approval.</t>
+          <t>CRISPR Therapeutics Q1 2026 results (released early May) showed Casgevy revenue of $43.0M with over 500 patients initiated globally, marking continued ramp of the first commercial CRISPR therapy; company holds $2.44B cash with multiple in vivo CRISPR INDs (CTX310, CTX460, CTX340) advancing.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260508584062/en/SkyWater-Technology-Stockholders-Approve-Merger-Agreement-with-IonQ | https://thequantuminsider.com/2026/05/09/skywater-technology-stockholders-approve-merger-agreement-with-ionq/</t>
+          <t>https://www.stocktitan.net/news/CRSP/crispr-therapeutics-provides-business-update-and-reports-first-sdrpmbu7dwil.html | https://ir.crisprtx.com/</t>
         </is>
       </c>
     </row>
@@ -10689,22 +10669,22 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>#10 Renewables + battery cost collapse</t>
+          <t>#08 Quantum error correction (logical qubits below threshold)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>CATL announces 40 GWh sodium-ion battery capacity expansion</t>
+          <t>IonQ-SkyWater $1.8B merger clears shareholder vote</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>On May 9, 2026, CATL disclosed via Ningde environmental authorities a 5B yuan ($735M) investment to add 40 GWh/year of sodium-ion power battery capacity at its Fuding Shidai subsidiary (24-month build); follows CATL's April three-year, 60 GWh sodium-ion supply contract with HyperStrong.</t>
+          <t>SkyWater Technology stockholders approved IonQ's ~$1.8B cash-and-stock acquisition at a May 8, 2026 special meeting (32.6M for, 405K against). Deal makes IonQ the only vertically integrated full-stack quantum platform with an in-house US semiconductor fab; closing expected Q2-Q3 2026 pending regulatory approval.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://cnevpost.com/2026/05/09/catl-plans-40-gwh-sodium-battery-capacity-expansion/</t>
+          <t>https://www.businesswire.com/news/home/20260508584062/en/SkyWater-Technology-Stockholders-Approve-Merger-Agreement-with-IonQ | https://thequantuminsider.com/2026/05/09/skywater-technology-stockholders-approve-merger-agreement-with-ionq/</t>
         </is>
       </c>
     </row>
@@ -10736,17 +10716,17 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>BNEF: global energy storage installs hit '100 GW era' in 2025</t>
+          <t>CATL announces 40 GWh sodium-ion battery capacity expansion</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>BloombergNEF's 1H 2026 Energy Storage Market Outlook (May 11, 2026) confirmed 112 GW / 307 GWh of new storage installed globally in 2025 — a 48% YoY jump and the first time the industry crossed 100 GW/year. BNEF forecasts 158 GW / 459 GWh in 2026 (+41%), with long-duration (6h+) storage additions set to quadruple to ~2 GW.</t>
+          <t>On May 9, 2026, CATL disclosed via Ningde environmental authorities a 5B yuan ($735M) investment to add 40 GWh/year of sodium-ion power battery capacity at its Fuding Shidai subsidiary (24-month build); follows CATL's April three-year, 60 GWh sodium-ion supply contract with HyperStrong.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>https://about.bnef.com/insights/clean-energy/energy-storage-enters-the-100-gigawatt-era-three-things-to-know/ | https://www.pv-magazine.com/2026/05/11/bloombergnef-confirms-energy-storage-has-reached-the-100-gw-era/</t>
+          <t>https://cnevpost.com/2026/05/09/catl-plans-40-gwh-sodium-battery-capacity-expansion/</t>
         </is>
       </c>
     </row>
@@ -10768,7 +10748,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>NEW_WATCH</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -10778,17 +10758,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Ford launches Ford Energy BESS subsidiary, 20 GWh/yr target</t>
+          <t>BNEF: global energy storage installs hit '100 GW era' in 2025</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>On May 11, 2026, Ford launched 'Ford Energy,' a US battery-energy-storage subsidiary repurposing the dissolved BlueOval SK plant in Glendale, KY to build LFP grid-scale storage for utilities, data centers, and industrial customers. Flagship FE-250 (2-hr) and FE-450 (4-hr) DC blocks use 512 Ah LFP prismatic cells; first deliveries late 2027; Lisa Drake named president.</t>
+          <t>BloombergNEF's 1H 2026 Energy Storage Market Outlook (May 11, 2026) confirmed 112 GW / 307 GWh of new storage installed globally in 2025 — a 48% YoY jump and the first time the industry crossed 100 GW/year. BNEF forecasts 158 GW / 459 GWh in 2026 (+41%), with long-duration (6h+) storage additions set to quadruple to ~2 GW.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://electrek.co/2026/05/11/ford-energy-launches-battery-storage-subsidiary-20gwh-bess/ | https://www.energy-storage.news/ford-officially-launches-us-stationary-energy-storage-subsidiary-deliveries-to-begin-in-2027/</t>
+          <t>https://about.bnef.com/insights/clean-energy/energy-storage-enters-the-100-gigawatt-era-three-things-to-know/ | https://www.pv-magazine.com/2026/05/11/bloombergnef-confirms-energy-storage-has-reached-the-100-gw-era/</t>
         </is>
       </c>
     </row>
@@ -10810,27 +10790,27 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
+          <t>NEW_WATCH</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>#15 AI accelerators / advanced compute</t>
+          <t>#10 Renewables + battery cost collapse</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Google adds Marvell as third TPU partner for inference + MPU</t>
+          <t>Ford launches Ford Energy BESS subsidiary, 20 GWh/yr target</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Reports on May 13, 2026 detailed Google co-developing two custom chips with Marvell: a memory processing unit (MPU) to pair with existing TPUs, and a next-gen inference-optimized TPU. Google plans nearly 2M MPUs, with design finalization expected in 2027 — diversifying beyond Broadcom and bringing MediaTek + Marvell into a four-partner TPU stack to challenge NVIDIA on inference economics.</t>
+          <t>On May 11, 2026, Ford launched 'Ford Energy,' a US battery-energy-storage subsidiary repurposing the dissolved BlueOval SK plant in Glendale, KY to build LFP grid-scale storage for utilities, data centers, and industrial customers. Flagship FE-250 (2-hr) and FE-450 (4-hr) DC blocks use 512 Ah LFP prismatic cells; first deliveries late 2027; Lisa Drake named president.</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>https://thenextweb.com/news/google-marvell-ai-chips-inference-tpu-broadcom | https://the-decoder.com/google-plans-nearly-two-million-new-ai-chips-as-it-turns-to-marvell-for-custom-designs/</t>
+          <t>https://electrek.co/2026/05/11/ford-energy-launches-battery-storage-subsidiary-20gwh-bess/ | https://www.energy-storage.news/ford-officially-launches-us-stationary-energy-storage-subsidiary-deliveries-to-begin-in-2027/</t>
         </is>
       </c>
     </row>
@@ -10852,23 +10832,27 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>BROAD_SCAN</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
+          <t>NEW_SUB_IDEA</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>#15 AI accelerators / advanced compute</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Archer Midnight enters UAE Restricted Type Certificate path (first eVTOL on RTC)</t>
+          <t>Google adds Marvell as third TPU partner for inference + MPU</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>On May 7-8, 2026, the UAE GCAA and Archer Aviation agreed to transition Midnight onto a Restricted Type Certificate (RTC) program, making Archer the first eVTOL maker on this streamlined pathway and opening the door to limited commercial air-taxi operations in Abu Dhabi.</t>
+          <t>Reports on May 13, 2026 detailed Google co-developing two custom chips with Marvell: a memory processing unit (MPU) to pair with existing TPUs, and a next-gen inference-optimized TPU. Google plans nearly 2M MPUs, with design finalization expected in 2027 — diversifying beyond Broadcom and bringing MediaTek + Marvell into a four-partner TPU stack to challenge NVIDIA on inference economics.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://investors.archer.com/news/news-details/2026/UAE-Regulator-And-Archer-Move-To-Streamlined-Approach-for-Certifying-Midnight-in-the-UAE/default.aspx | https://www.flightglobal.com/airframers/2026/05/archers-uae-restricted-type-certificate-plan-poses-questions-over-operational-limitations/</t>
+          <t>https://thenextweb.com/news/google-marvell-ai-chips-inference-tpu-broadcom | https://the-decoder.com/google-plans-nearly-two-million-new-ai-chips-as-it-turns-to-marvell-for-custom-designs/</t>
         </is>
       </c>
     </row>
@@ -10896,17 +10880,17 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>EU agrees AI Act 'omnibus' simplification; nudification ban added</t>
+          <t>Archer Midnight enters UAE Restricted Type Certificate path (first eVTOL on RTC)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>On May 7, 2026 the Council and Parliament reached political agreement on the AI Act omnibus, delaying national sandbox deadlines to August 2027, shortening transparency grace periods, and adding a ban on 'nudification' apps. Commission followed May 8 with draft transparency guidelines — reshaping the EU AI governance timeline before the August 2026 GPAI enforcement date.</t>
+          <t>On May 7-8, 2026, the UAE GCAA and Archer Aviation agreed to transition Midnight onto a Restricted Type Certificate (RTC) program, making Archer the first eVTOL maker on this streamlined pathway and opening the door to limited commercial air-taxi operations in Abu Dhabi.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>https://www.consilium.europa.eu/en/press/press-releases/2026/05/07/artificial-intelligence-council-and-parliament-agree-to-simplify-and-streamline-rules/ | https://www.lw.com/en/insights/ai-act-update-eu-resolves-to-change-rules-and-extend-deadlines</t>
+          <t>https://investors.archer.com/news/news-details/2026/UAE-Regulator-And-Archer-Move-To-Streamlined-Approach-for-Certifying-Midnight-in-the-UAE/default.aspx | https://www.flightglobal.com/airframers/2026/05/archers-uae-restricted-type-certificate-plan-poses-questions-over-operational-limitations/</t>
         </is>
       </c>
     </row>
@@ -10934,24 +10918,24 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>HKU 'SS-H2' super-stainless steel could cut green-H2 structural costs ~40x</t>
+          <t>EU agrees AI Act 'omnibus' simplification; nudification ban added</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Reported May 10-11, 2026: a University of Hong Kong team led by Mingxin Huang published a 'sequential dual-passivation' stainless steel (SS-H2) that resists corrosion at ultra-high potentials in seawater electrolysis, potentially replacing titanium components and slashing structural costs ~40-fold for seawater green-hydrogen.</t>
+          <t>On May 7, 2026 the Council and Parliament reached political agreement on the AI Act omnibus, delaying national sandbox deadlines to August 2027, shortening transparency grace periods, and adding a ban on 'nudification' apps. Commission followed May 8 with draft transparency guidelines — reshaping the EU AI governance timeline before the August 2026 GPAI enforcement date.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://www.sciencedaily.com/releases/2026/05/260510030950.htm | https://fuelcellsworks.com/2026/05/11/clean-energy/cannot-be-explained-new-ultra-stainless-steel-stuns-researchers</t>
+          <t>https://www.consilium.europa.eu/en/press/press-releases/2026/05/07/artificial-intelligence-council-and-parliament-agree-to-simplify-and-streamline-rules/ | https://www.lw.com/en/insights/ai-act-update-eu-resolves-to-change-rules-and-extend-deadlines</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -10961,32 +10945,28 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Intra-day supplement to the morning's run: three primary-source items the AM scan missed. Anthropic took all of SpaceX's Colossus 1 (May 6) — 300+ MW / 220K+ NVIDIA GPUs immediately, plus stated interest in multi-GW orbital compute — and used the new headroom to double Claude Code rate limits and raise Opus API limits. Anthropic Interpretability published Natural Language Autoencoders (May 7), an unsupervised method that translates Claude's residual-stream activations into readable text and was already used in the Mythos Preview and Opus 4.6 alignment audits. OpenAI opened GPT-5.5-Cyber to vetted defenders via Trusted Access for Cyber (May 7), the most-permissive cyber variant yet, with Cisco and CrowdStrike as launch partners.</t>
+          <t>Heavy commercialization week across bio and AI infrastructure. In bio: Isomorphic Labs closed a $2.1B Series B led by Thrive Capital — one of the largest private AI-drug-discovery rounds on record — while Intellia opened a rolling BLA for lonvo-z (first-ever in vivo CRISPR product, US launch tracking H1 2027), Editas reported &gt;=90% LDL-C reduction in NHPs for EDIT-401 at ASGCT, Viking presented 12.2% 13-week weight loss for oral VK2735 at ECO 2026, and Neuralink signaled a next-gen 'whole-brain' surgical robot. In AI/robotics: Waymo expanded to 1,400 sq mi across 11 metros (FIFA World Cup readiness), Figure ran a full 8-hour fully autonomous package-sorting shift on Helix-02, China's ROBOTERA closed &gt;$200M led by SF Group, and Google launched Gemini Intelligence as an OS-level agent for Android. Energy/quantum: CATL announced a 40 GWh sodium-ion expansion, BNEF confirmed energy storage entered the '100 GW era' in 2025, Ford launched a 20 GWh/yr LFP grid-storage subsidiary, IonQ shareholders approved the $1.8B SkyWater acquisition, and Google added Marvell as a third TPU partner targeting ~2M inference MPUs. Agent D flagged three adjacencies: Archer's UAE Restricted Type Certificate path (first eVTOL on this pathway), the EU AI Act omnibus simplification (and nudification ban), and an HKU ultra-stainless-steel claim that could cut seawater-electrolysis structural costs ~40x.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>#01 Transformers / LLMs / coding agents</t>
-        </is>
-      </c>
+          <t>BROAD_SCAN</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Anthropic + SpaceX Colossus 1 deal: 300+ MW / 220K+ GPUs in a month</t>
+          <t>HKU 'SS-H2' super-stainless steel could cut green-H2 structural costs ~40x</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Anthropic signed for the entire compute capacity of SpaceX's Colossus 1 data center in Memphis — 300+ MW (over 220,000 NVIDIA GPUs) coming online within the month — and immediately doubled Claude Code five-hour rate limits and raised Opus API limits; the agreement also includes stated interest in multi-gigawatt orbital AI compute with SpaceX.</t>
+          <t>Reported May 10-11, 2026: a University of Hong Kong team led by Mingxin Huang published a 'sequential dual-passivation' stainless steel (SS-H2) that resists corrosion at ultra-high potentials in seawater electrolysis, potentially replacing titanium components and slashing structural costs ~40-fold for seawater green-hydrogen.</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/news/higher-limits-spacex | https://www.cnbc.com/2026/05/06/anthropic-spacex-data-center-capacity.html | https://www.bloomberg.com/news/articles/2026-05-06/anthropic-inks-computing-deal-with-spacex-to-meet-ai-demand</t>
+          <t>https://www.sciencedaily.com/releases/2026/05/260510030950.htm | https://fuelcellsworks.com/2026/05/11/clean-energy/cannot-be-explained-new-ultra-stainless-steel-stuns-researchers</t>
         </is>
       </c>
     </row>
@@ -11013,22 +10993,22 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>#02 RLHF + reasoning models (test-time compute scaling)</t>
+          <t>#01 Transformers / LLMs / coding agents</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Natural Language Autoencoders read Claude's activations as text</t>
+          <t>Anthropic + SpaceX Colossus 1 deal: 300+ MW / 220K+ GPUs in a month</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Anthropic Interpretability released Natural Language Autoencoders (NLAs) — verbalizer/reconstructor LLM pair, RL-trained for round-trip activation→text→activation fidelity — that surface unverbalized evaluation-awareness on 16-26% of safety/SWE-bench transcripts (vs &lt;1% on real opt-in usage) and lift hidden-motivation auditing from &lt;3% to 12-15%; deployed in Mythos Preview and Opus 4.6 pre-deployment audits, with code and Neuronpedia frontend released.</t>
+          <t>Anthropic signed for the entire compute capacity of SpaceX's Colossus 1 data center in Memphis — 300+ MW (over 220,000 NVIDIA GPUs) coming online within the month — and immediately doubled Claude Code five-hour rate limits and raised Opus API limits; the agreement also includes stated interest in multi-gigawatt orbital AI compute with SpaceX.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/research/natural-language-autoencoders | https://transformer-circuits.pub/2026/nla/index.html | https://github.com/kitft/natural_language_autoencoders</t>
+          <t>https://www.anthropic.com/news/higher-limits-spacex | https://www.cnbc.com/2026/05/06/anthropic-spacex-data-center-capacity.html | https://www.bloomberg.com/news/articles/2026-05-06/anthropic-inks-computing-deal-with-spacex-to-meet-ai-demand</t>
         </is>
       </c>
     </row>
@@ -11050,27 +11030,27 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>#01 Transformers / LLMs / coding agents</t>
+          <t>#02 RLHF + reasoning models (test-time compute scaling)</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>OpenAI GPT-5.5-Cyber via Trusted Access for Cyber program</t>
+          <t>Anthropic Natural Language Autoencoders read Claude's activations as text</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>OpenAI rolled out GPT-5.5-Cyber, the most-permissive variant of GPT-5.5 for vetted security defenders (bug-hunting, malware analysis, reverse engineering allowed; credential-theft and malware-writing still blocked), gated via Trusted Access for Cyber identity tier with Cisco and CrowdStrike among the launch partners; Axios sources put offensive-cyber capability roughly on par with Anthropic Mythos Preview.</t>
+          <t>Anthropic Interpretability released Natural Language Autoencoders (NLAs) — verbalizer/reconstructor LLM pair, RL-trained for round-trip activation→text→activation fidelity — that surface unverbalized evaluation-awareness on 16-26% of safety/SWE-bench transcripts (vs &lt;1% on real opt-in usage) and lift hidden-motivation auditing from &lt;3% to 12-15%; deployed in Mythos Preview and Opus 4.6 pre-deployment audits, with code and Neuronpedia frontend released.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>https://openai.com/index/gpt-5-5-with-trusted-access-for-cyber/ | https://www.cnbc.com/2026/05/07/openai-rolls-out-new-gpt-5point5-cyber-to-vetted-cybersecurity-teams.html | https://www.axios.com/2026/05/07/openai-gpt-55-cybersecurity-model</t>
+          <t>https://www.anthropic.com/research/natural-language-autoencoders | https://transformer-circuits.pub/2026/nla/index.html | https://github.com/kitft/natural_language_autoencoders</t>
         </is>
       </c>
     </row>
@@ -11087,12 +11067,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Heavy week across AI infra, AI hardware, quantum, and bio. OpenAI shipped GPT-5.5 Instant (52.5% hallucination reduction) and a new GPT-Realtime-2 voice stack; Anthropic stood up a $1.5B enterprise-AI JV with Blackstone, H&amp;F, and Goldman; Allen Institute released MolmoAct2 (open bimanual VLA) and Figure ramped Figure 03 to roughly 1 robot/hour. Cerebras filed for a $26.6B IPO with a multi-year OpenAI compute deal, and IBM marked a decade of cloud-quantum while quantum-simulating a 12,635-atom protein with Cleveland Clinic + RIKEN. In bio, Isomorphic Labs published its IsoDDE drug-design engine doubling AlphaFold 3 protein-ligand accuracy, Synchron became the first BCI to land native Apple HID integration, and AACR readouts showed personalized neoantigen mRNA vaccines durable in pancreatic Phase 1. In space and energy, Rocket Lab booked a record multi-Neutron deal and Zap Energy pivoted to a hybrid fission-fusion strategy. Agent D's broad scan returned a Joby Manhattan eVTOL demo and Fervo's $1.33B geothermal IPO filing.</t>
+          <t>Intra-day supplement to the morning's run: three primary-source items the AM scan missed. Anthropic took all of SpaceX's Colossus 1 (May 6) — 300+ MW / 220K+ NVIDIA GPUs immediately, plus stated interest in multi-GW orbital compute — and used the new headroom to double Claude Code rate limits and raise Opus API limits. Anthropic Interpretability published Natural Language Autoencoders (May 7), an unsupervised method that translates Claude's residual-stream activations into readable text and was already used in the Mythos Preview and Opus 4.6 alignment audits. OpenAI opened GPT-5.5-Cyber to vetted defenders via Trusted Access for Cyber (May 7), the most-permissive cyber variant yet, with Cisco and CrowdStrike as launch partners.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>NEW_SUB_IDEA</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -11102,17 +11082,17 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>OpenAI GPT-5.5 Instant: 52.5% hallucination reduction</t>
+          <t>OpenAI GPT-5.5-Cyber via Trusted Access for Cyber program</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>OpenAI released GPT-5.5 Instant on May 5 as the new default ChatGPT model with personalized search; benchmarks show 52.5% fewer hallucinated claims than GPT-5.3 Instant on medicine, law, and finance prompts.</t>
+          <t>OpenAI rolled out GPT-5.5-Cyber, the most-permissive variant of GPT-5.5 for vetted security defenders (bug-hunting, malware analysis, reverse engineering allowed; credential-theft and malware-writing still blocked), gated via Trusted Access for Cyber identity tier with Cisco and CrowdStrike among the launch partners; Axios sources put offensive-cyber capability roughly on par with Anthropic Mythos Preview.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://openai.com/index/gpt-5-5-instant/</t>
+          <t>https://openai.com/index/gpt-5-5-with-trusted-access-for-cyber/ | https://www.cnbc.com/2026/05/07/openai-rolls-out-new-gpt-5point5-cyber-to-vetted-cybersecurity-teams.html | https://www.axios.com/2026/05/07/openai-gpt-55-cybersecurity-model</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11114,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -11144,17 +11124,17 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>OpenAI Realtime-2 voice stack: GPT-5-class reasoning over audio</t>
+          <t>OpenAI GPT-5.5 Instant: 52.5% hallucination reduction</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>OpenAI launched three audio models on May 7: GPT-Realtime-2 (GPT-5-class voice reasoning, +15.2% on Big Bench Audio), GPT-Realtime-Translate (70+ languages), and GPT-Realtime-Whisper (streaming transcription).</t>
+          <t>OpenAI released GPT-5.5 Instant on May 5 as the new default ChatGPT model with personalized search; benchmarks show 52.5% fewer hallucinated claims than GPT-5.3 Instant on medicine, law, and finance prompts.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>https://openai.com/index/advancing-voice-intelligence-with-new-models-in-the-api/</t>
+          <t>https://openai.com/index/gpt-5-5-instant/</t>
         </is>
       </c>
     </row>
@@ -11176,7 +11156,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>NEW_WATCH</t>
+          <t>NEW_SUB_IDEA</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -11186,17 +11166,17 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Anthropic + Blackstone/H&amp;F/Goldman launch $1.5B enterprise-AI JV</t>
+          <t>OpenAI Realtime-2 voice stack: GPT-5-class reasoning over audio</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Anthropic announced (May 4) a $1.5B-capitalized joint venture with Blackstone, Hellman &amp; Friedman, and Goldman Sachs to build a services company embedding Claude in mid-market enterprises.</t>
+          <t>OpenAI launched three audio models on May 7: GPT-Realtime-2 (GPT-5-class voice reasoning, +15.2% on Big Bench Audio), GPT-Realtime-Translate (70+ languages), and GPT-Realtime-Whisper (streaming transcription).</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/news/enterprise-ai-services-company</t>
+          <t>https://openai.com/index/advancing-voice-intelligence-with-new-models-in-the-api/</t>
         </is>
       </c>
     </row>
@@ -11218,27 +11198,27 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>NEW_WATCH</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>#02 RLHF + reasoning models (test-time compute scaling)</t>
+          <t>#01 Transformers / LLMs / coding agents</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>TraceLift: executor-grounded reasoning rewards via downstream uplift</t>
+          <t>Anthropic + Blackstone/H&amp;F/Goldman launch $1.5B enterprise-AI JV</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>arXiv 2605.03862 (May 5) proposes TraceLift, which scores reasoning traces by both rubric-based reward-model quality and measured uplift on frozen downstream executors, crediting traces that are useful, not just well-formed.</t>
+          <t>Anthropic announced (May 4) a $1.5B-capitalized joint venture with Blackstone, Hellman &amp; Friedman, and Goldman Sachs to build a services company embedding Claude in mid-market enterprises.</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.03862</t>
+          <t>https://www.anthropic.com/news/enterprise-ai-services-company</t>
         </is>
       </c>
     </row>
@@ -11260,27 +11240,27 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>#12 Humanoid robotics</t>
+          <t>#02 RLHF + reasoning models (test-time compute scaling)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Allen Institute MolmoAct2: open bimanual VLA model</t>
+          <t>TraceLift: executor-grounded reasoning rewards via downstream uplift</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>AI2 released MolmoAct2 (May 5) - an open-source Vision-Language-Action model trained on 720 hours of bimanual teleoperation, reporting 87.1% success on real-world DROID tasks with unseen objects and ~37x faster inference than its predecessor.</t>
+          <t>arXiv 2605.03862 (May 5) proposes TraceLift, which scores reasoning traces by both rubric-based reward-model quality and measured uplift on frozen downstream executors, crediting traces that are useful, not just well-formed.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://allenai.org/blog/molmoact2 | https://arxiv.org/abs/2605.02881</t>
+          <t>https://arxiv.org/abs/2605.03862</t>
         </is>
       </c>
     </row>
@@ -11302,7 +11282,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>NEW_WATCH</t>
+          <t>NEW_SUB_IDEA</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -11312,17 +11292,17 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Figure 03 production hits 1 robot/hour, Helix S0 ditches teleop</t>
+          <t>Allen Institute MolmoAct2: open bimanual VLA model</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Figure AI announced (May 1) ramping Figure 03 to ~1 robot/hour (vs 1/day four months prior); 350+ units produced and Helix S0 now handles stairs and uneven terrain without teleoperation.</t>
+          <t>AI2 released MolmoAct2 (May 5) - an open-source Vision-Language-Action model trained on 720 hours of bimanual teleoperation, reporting 87.1% success on real-world DROID tasks with unseen objects and ~37x faster inference than its predecessor.</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>https://www.figure.ai/news/ramping-figure-03-production | https://theaiinsider.tech/2026/05/01/figure-ai-ramps-up-production-to-one-humanoid-robot-per-hour/</t>
+          <t>https://allenai.org/blog/molmoact2 | https://arxiv.org/abs/2605.02881</t>
         </is>
       </c>
     </row>
@@ -11344,27 +11324,27 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>NEW_WATCH</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>#04 AlphaFold + computational protein design</t>
+          <t>#12 Humanoid robotics</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Isomorphic Labs IsoDDE doubles AlphaFold 3 on protein-ligand prediction</t>
+          <t>Figure 03 production hits 1 robot/hour, Helix S0 ditches teleop</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Isomorphic Labs published the Isomorphic Drug Design Engine (IsoDDE), reporting ~50% accuracy on hard low-sequence-identity protein-ligand cases vs ~23% for AlphaFold 3, plus prediction of cryptic binding sites and small-molecule affinities.</t>
+          <t>Figure AI announced (May 1) ramping Figure 03 to ~1 robot/hour (vs 1/day four months prior); 350+ units produced and Helix S0 now handles stairs and uneven terrain without teleoperation.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://www.isomorphiclabs.com/articles/the-isomorphic-labs-drug-design-engine-unlocks-a-new-frontier</t>
+          <t>https://www.figure.ai/news/ramping-figure-03-production | https://theaiinsider.tech/2026/05/01/figure-ai-ramps-up-production-to-one-humanoid-robot-per-hour/</t>
         </is>
       </c>
     </row>
@@ -11391,22 +11371,22 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>#14 Brain-computer interfaces</t>
+          <t>#04 AlphaFold + computational protein design</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Synchron is first BCI with native Apple HID input integration</t>
+          <t>Isomorphic Labs IsoDDE doubles AlphaFold 3 on protein-ligand prediction</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Synchron announced native integration with Apple's BCI HID profile, becoming the first BCI company recognized as a native Apple input category - enabling hands-free device control for ALS and spinal-cord-injury patients.</t>
+          <t>Isomorphic Labs published the Isomorphic Drug Design Engine (IsoDDE), reporting ~50% accuracy on hard low-sequence-identity protein-ligand cases vs ~23% for AlphaFold 3, plus prediction of cryptic binding sites and small-molecule affinities.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>https://www.medicaleconomics.com/view/synchron-first-to-integrate-brain-computer-interface-with-apple-devices</t>
+          <t>https://www.isomorphiclabs.com/articles/the-isomorphic-labs-drug-design-engine-unlocks-a-new-frontier</t>
         </is>
       </c>
     </row>
@@ -11428,27 +11408,27 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>#05 mRNA vaccines + LNP delivery</t>
+          <t>#14 Brain-computer interfaces</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>AACR 2026: personalized neoantigen mRNA vaccines hit ~90% survival in pancreatic Phase 1</t>
+          <t>Synchron is first BCI with native Apple HID input integration</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>AACR May 2026 readouts and a Mount Sinai review highlighted personalized neoantigen mRNA vaccines: autogene cevumeran (BioNTech/Roche) showing ~90% 6-year survival in pancreatic Phase 1 with checkpoint inhibitor; mRNA-4157 (Moderna/Merck) advancing in Phase 3.</t>
+          <t>Synchron announced native integration with Apple's BCI HID profile, becoming the first BCI company recognized as a native Apple input category - enabling hands-free device control for ALS and spinal-cord-injury patients.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://www.mountsinai.org/about/newsroom/2026/mount-sinai-review-maps-the-path-forward-for-cancer-vaccines-highlighting-promise-of-personalized-and-combination-approaches</t>
+          <t>https://www.medicaleconomics.com/view/synchron-first-to-integrate-brain-computer-interface-with-apple-devices</t>
         </is>
       </c>
     </row>
@@ -11470,27 +11450,27 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_SUB_IDEA</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>#08 Quantum error correction (logical qubits below threshold)</t>
+          <t>#05 mRNA vaccines + LNP delivery</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>IBM + Cleveland Clinic + RIKEN simulate 12,635-atom protein on quantum hardware</t>
+          <t>AACR 2026: personalized neoantigen mRNA vaccines hit ~90% survival in pancreatic Phase 1</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>IBM, Cleveland Clinic, and RIKEN announced (May 5) a quantum-centric supercomputing simulation of trypsin (12,635 atoms) using 156-qubit Heron processors - a ~40x increase in simulated system size in six months.</t>
+          <t>AACR May 2026 readouts and a Mount Sinai review highlighted personalized neoantigen mRNA vaccines: autogene cevumeran (BioNTech/Roche) showing ~90% 6-year survival in pancreatic Phase 1 with checkpoint inhibitor; mRNA-4157 (Moderna/Merck) advancing in Phase 3.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>https://newsroom.ibm.com/2026-05-05-cleveland-clinic,-riken,-and-ibm-model-a-12,635-atom-protein-the-largest-known-to-be-simulated-with-quantum-computers</t>
+          <t>https://www.mountsinai.org/about/newsroom/2026/mount-sinai-review-maps-the-path-forward-for-cancer-vaccines-highlighting-promise-of-personalized-and-combination-approaches</t>
         </is>
       </c>
     </row>
@@ -11522,17 +11502,17 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>IBM marks 10 years of cloud-accessible quantum computing</t>
+          <t>IBM + Cleveland Clinic + RIKEN simulate 12,635-atom protein on quantum hardware</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>IBM (May 4) marked the decade since the first cloud-accessible quantum processor, now operating 156-qubit Heron systems with ~1.17e-3 median two-qubit error rate.</t>
+          <t>IBM, Cleveland Clinic, and RIKEN announced (May 5) a quantum-centric supercomputing simulation of trypsin (12,635 atoms) using 156-qubit Heron processors - a ~40x increase in simulated system size in six months.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://newsroom.ibm.com/2026-05-04-ibm-a-decade-of-quantum-on-the-cloud</t>
+          <t>https://newsroom.ibm.com/2026-05-05-cleveland-clinic,-riken,-and-ibm-model-a-12,635-atom-protein-the-largest-known-to-be-simulated-with-quantum-computers</t>
         </is>
       </c>
     </row>
@@ -11554,27 +11534,27 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>#15 AI accelerators / advanced compute</t>
+          <t>#08 Quantum error correction (logical qubits below threshold)</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Cerebras files $3.5B IPO at $26.6B with multi-year OpenAI compute deal</t>
+          <t>IBM marks 10 years of cloud-accessible quantum computing</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Cerebras filed its S-1 (May 4) targeting $115-125/share at a ~$26.6B valuation, anchored by a $20B+ multi-year OpenAI co-design and inference compute deal; FY25 revenue $510M (+76% YoY).</t>
+          <t>IBM (May 4) marked the decade since the first cloud-accessible quantum processor, now operating 156-qubit Heron systems with ~1.17e-3 median two-qubit error rate.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/05/04/openais-cozy-partner-cerebras-is-on-track-for-a-blockbuster-ipo/ | https://www.cnbc.com/2026/05/04/cerebras-ipo-ai-chipmaker.html</t>
+          <t>https://newsroom.ibm.com/2026-05-04-ibm-a-decade-of-quantum-on-the-cloud</t>
         </is>
       </c>
     </row>
@@ -11596,27 +11576,27 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>NEW_WATCH</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>#09 Reusable rockets (Falcon 9 + Starship catch)</t>
+          <t>#15 AI accelerators / advanced compute</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Rocket Lab books multi-Neutron deal; backlog past $2.2B</t>
+          <t>Cerebras files $3.5B IPO at $26.6B with multi-year OpenAI compute deal</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Rocket Lab (May 7) reported Q1 2026 revenue +63.5% YoY to $200M and announced a confidential customer's multi-launch Neutron + Electron deal; backlog now exceeds $2.2B with Neutron's Q4 2026 debut on track.</t>
+          <t>Cerebras filed its S-1 (May 4) targeting $115-125/share at a ~$26.6B valuation, anchored by a $20B+ multi-year OpenAI co-design and inference compute deal; FY25 revenue $510M (+76% YoY).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://spaceflightnow.com/2026/05/07/rocket-lab-announces-five-launch-neutron-deal-as-it-continues-aiming-for-late-2026-debut/ | https://www.globenewswire.com/news-release/2026/05/07/3290605/0/en/rocket-lab-s-biggest-launch-deal-yet-confidential-customer-books-multiple-neutron-and-electron-launches.html</t>
+          <t>https://techcrunch.com/2026/05/04/openais-cozy-partner-cerebras-is-on-track-for-a-blockbuster-ipo/ | https://www.cnbc.com/2026/05/04/cerebras-ipo-ai-chipmaker.html</t>
         </is>
       </c>
     </row>
@@ -11638,27 +11618,27 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_WATCH</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>#13 Fusion energy</t>
+          <t>#09 Reusable rockets (Falcon 9 + Starship catch)</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Zap Energy announces industry-first hybrid fission-fusion strategy</t>
+          <t>Rocket Lab books multi-Neutron deal; backlog past $2.2B</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Zap Energy (May 5) announced plans to develop small-scale nuclear fission alongside its z-pinch fusion platform - an industry first - and named Zabrina Johal as CEO; ranked #16 on TIME/Statista GreenTech 2026.</t>
+          <t>Rocket Lab (May 7) reported Q1 2026 revenue +63.5% YoY to $200M and announced a confidential customer's multi-launch Neutron + Electron deal; backlog now exceeds $2.2B with Neutron's Q4 2026 debut on track.</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>https://www.nucnet.org/news/in-an-industry-first-zap-energy-adds-fusion-to-traditional-fission-lineup-5-5-2026 | https://www.realclearenergy.org/articles/2026/05/04/zap_energy_the_first_fission-fusion_company_1180637.html</t>
+          <t>https://spaceflightnow.com/2026/05/07/rocket-lab-announces-five-launch-neutron-deal-as-it-continues-aiming-for-late-2026-debut/ | https://www.globenewswire.com/news-release/2026/05/07/3290605/0/en/rocket-lab-s-biggest-launch-deal-yet-confidential-customer-books-multiple-neutron-and-electron-launches.html</t>
         </is>
       </c>
     </row>
@@ -11680,23 +11660,27 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>BROAD_SCAN</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr"/>
+          <t>UPDATED_FACT</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>#13 Fusion energy</t>
+        </is>
+      </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Joby flies passenger-style eVTOL demo over Manhattan at 45 dB cruise</t>
+          <t>Zap Energy announces industry-first hybrid fission-fusion strategy</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Joby Aviation (May 1) ran a public eVTOL demo at NYC's East 34th Street Heliport, flying a passenger-style sortie at ~45 dB cruise noise and proving urban-infrastructure compatibility for sub-10-minute cross-city hops.</t>
+          <t>Zap Energy (May 5) announced plans to develop small-scale nuclear fission alongside its z-pinch fusion platform - an industry first - and named Zabrina Johal as CEO; ranked #16 on TIME/Statista GreenTech 2026.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/01/3286156/0/en/VertiPorts-by-Atlantic-Hosts-Electric-Air-Taxi-Demonstration-by-Joby-Aviation-at-New-York-City-s-East-34th-Street-Heliport.html</t>
+          <t>https://www.nucnet.org/news/in-an-industry-first-zap-energy-adds-fusion-to-traditional-fission-lineup-5-5-2026 | https://www.realclearenergy.org/articles/2026/05/04/zap_energy_the_first_fission-fusion_company_1180637.html</t>
         </is>
       </c>
     </row>
@@ -11724,17 +11708,17 @@
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Fervo Energy files $1.33B IPO; Cape Station EGS targeting 500 MW by 2028</t>
+          <t>Joby flies passenger-style eVTOL demo over Manhattan at 45 dB cruise</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Fervo Energy filed for a $1.33B IPO (May 4) with its Cape Station enhanced-geothermal plant tracking first-power in October 2026 and a 500 MW build-out by 2028, at ~$7k/kW capex (target $3k/kW).</t>
+          <t>Joby Aviation (May 1) ran a public eVTOL demo at NYC's East 34th Street Heliport, flying a passenger-style sortie at ~45 dB cruise noise and proving urban-infrastructure compatibility for sub-10-minute cross-city hops.</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>https://www.bloomberg.com/news/articles/2026-05-04/geothermal-energy-developer-fervo-seeks-1-33-billion-in-us-ipo</t>
+          <t>https://www.globenewswire.com/news-release/2026/05/01/3286156/0/en/VertiPorts-by-Atlantic-Hosts-Electric-Air-Taxi-Demonstration-by-Joby-Aviation-at-New-York-City-s-East-34th-Street-Heliport.html</t>
         </is>
       </c>
     </row>
@@ -11751,32 +11735,28 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Quietly busy week dominated by AI-tooling, quantum, and clinical-bio progress. AWS shipped a managed MCP server for AWS APIs; three reasoning-RL papers hit arXiv (sparse-policy, scaling-exponent, and search-driven reward optimization); QuEra/Harvard/MIT demonstrated a 2:1 physical-to-logical qubit ratio and NVIDIA released open AI models for QEC decoding/calibration; CRISPR Therapeutics reported $43M Q1 Casgevy revenue with 500+ patients on therapy; Neuralink unveiled a high-throughput automated implant robot; and IRENA published an updated outlook showing firm 24/7 solar+storage at $54-82/MWh.</t>
+          <t>Heavy week across AI infra, AI hardware, quantum, and bio. OpenAI shipped GPT-5.5 Instant (52.5% hallucination reduction) and a new GPT-Realtime-2 voice stack; Anthropic stood up a $1.5B enterprise-AI JV with Blackstone, H&amp;F, and Goldman; Allen Institute released MolmoAct2 (open bimanual VLA) and Figure ramped Figure 03 to roughly 1 robot/hour. Cerebras filed for a $26.6B IPO with a multi-year OpenAI compute deal, and IBM marked a decade of cloud-quantum while quantum-simulating a 12,635-atom protein with Cleveland Clinic + RIKEN. In bio, Isomorphic Labs published its IsoDDE drug-design engine doubling AlphaFold 3 protein-ligand accuracy, Synchron became the first BCI to land native Apple HID integration, and AACR readouts showed personalized neoantigen mRNA vaccines durable in pancreatic Phase 1. In space and energy, Rocket Lab booked a record multi-Neutron deal and Zap Energy pivoted to a hybrid fission-fusion strategy. Agent D's broad scan returned a Joby Manhattan eVTOL demo and Fervo's $1.33B geothermal IPO filing.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>#01 Transformers / LLMs / coding agents</t>
-        </is>
-      </c>
+          <t>BROAD_SCAN</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>AWS MCP Server reaches GA with managed agent access to AWS APIs</t>
+          <t>Fervo Energy files $1.33B IPO; Cape Station EGS targeting 500 MW by 2028</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>AWS launched a managed MCP server (May 6, 2026) letting coding agents call any AWS API via a single tool, with IAM guardrails, CloudTrail logging, and sandboxed Python execution.</t>
+          <t>Fervo Energy filed for a $1.33B IPO (May 4) with its Cape Station enhanced-geothermal plant tracking first-power in October 2026 and a 500 MW build-out by 2028, at ~$7k/kW capex (target $3k/kW).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>https://aws.amazon.com/blogs/aws/the-aws-mcp-server-is-now-generally-available/ | https://aws.amazon.com/about-aws/whats-new/2026/05/aws-mcp-server/</t>
+          <t>https://www.bloomberg.com/news/articles/2026-05-04/geothermal-energy-developer-fervo-seeks-1-33-billion-in-us-ipo</t>
         </is>
       </c>
     </row>
@@ -11798,27 +11778,27 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>NEW_SUB_IDEA</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>#02 RLHF + reasoning models (test-time compute scaling)</t>
+          <t>#01 Transformers / LLMs / coding agents</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Sparse policy selection rivals full RL on reasoning at 1000x lower compute</t>
+          <t>AWS MCP Server reaches GA with managed agent access to AWS APIs</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>ReasonMaxxer paper claims entropy-gated contrastive loss matches or exceeds full-RL reasoning performance with three orders of magnitude less training compute.</t>
+          <t>AWS launched a managed MCP server (May 6, 2026) letting coding agents call any AWS API via a single tool, with IAM guardrails, CloudTrail logging, and sandboxed Python execution.</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.06241</t>
+          <t>https://aws.amazon.com/blogs/aws/the-aws-mcp-server-is-now-generally-available/ | https://aws.amazon.com/about-aws/whats-new/2026/05/aws-mcp-server/</t>
         </is>
       </c>
     </row>
@@ -11850,17 +11830,17 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Scaling exponent for RL reasoning grows with logical expressiveness</t>
+          <t>Sparse policy selection rivals full RL on reasoning at 1000x lower compute</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>ScaleLogic shows RL training compute follows a power law with reasoning depth, with the exponent rising from 1.04 to 2.60 as logical expressiveness increases.</t>
+          <t>ReasonMaxxer paper claims entropy-gated contrastive loss matches or exceeds full-RL reasoning performance with three orders of magnitude less training compute.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.06638</t>
+          <t>https://arxiv.org/abs/2605.06241</t>
         </is>
       </c>
     </row>
@@ -11892,17 +11872,17 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Search-driven reward optimization improves reasoning without retraining</t>
+          <t>Scaling exponent for RL reasoning grows with logical expressiveness</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>New framework treats reward specification as an optimization object: it generates candidate reward functions, validates them automatically, and ranks them on GSM8K without modifying the base model.</t>
+          <t>ScaleLogic shows RL training compute follows a power law with reasoning depth, with the exponent rising from 1.04 to 2.60 as logical expressiveness increases.</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.02073</t>
+          <t>https://arxiv.org/abs/2605.06638</t>
         </is>
       </c>
     </row>
@@ -11924,27 +11904,27 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>#07 CRISPR therapies (Casgevy + base/prime editing)</t>
+          <t>#02 RLHF + reasoning models (test-time compute scaling)</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Casgevy Q1 2026: $43M revenue, 500+ patients on therapy</t>
+          <t>Search-driven reward optimization improves reasoning without retraining</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>CRISPR Therapeutics' May 4 business update reported $43M of Casgevy revenue in Q1 2026 and over 500 patients initiated, with continued progress on zugo-cel in autoimmune indications and in vivo liver-directed programs.</t>
+          <t>New framework treats reward specification as an optimization object: it generates candidate reward functions, validates them automatically, and ranks them on GSM8K without modifying the base model.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/04/3287176/0/en/CRISPR-Therapeutics-Provides-Business-Update-and-Reports-First-Quarter-2026-Financial-Results.html</t>
+          <t>https://arxiv.org/abs/2605.02073</t>
         </is>
       </c>
     </row>
@@ -11966,27 +11946,27 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>#14 Brain-computer interfaces</t>
+          <t>#07 CRISPR therapies (Casgevy + base/prime editing)</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Neuralink unveils automated high-throughput surgical robot</t>
+          <t>Casgevy Q1 2026: $43M revenue, 500+ patients on therapy</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Neuralink (May 7, 2026) outlined plans for high-volume BCI production paired with a streamlined, largely automated implantation procedure, with the robot accessing arbitrary cortical targets via threads through the dura.</t>
+          <t>CRISPR Therapeutics' May 4 business update reported $43M of Casgevy revenue in Q1 2026 and over 500 patients initiated, with continued progress on zugo-cel in autoimmune indications and in vivo liver-directed programs.</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>https://x.com/elonmusk/status/2006513491105165411 | https://yourstory.com/2026/05/neuralink-surgical-robot-brain-interface-2026</t>
+          <t>https://www.globenewswire.com/news-release/2026/05/04/3287176/0/en/CRISPR-Therapeutics-Provides-Business-Update-and-Reports-First-Quarter-2026-Financial-Results.html</t>
         </is>
       </c>
     </row>
@@ -12008,27 +11988,27 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>NEW_SUB_IDEA</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>#05 mRNA vaccines + LNP delivery</t>
+          <t>#14 Brain-computer interfaces</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Reduced-reactogenicity LNP-mRNA design preserves antibody response</t>
+          <t>Neuralink unveils automated high-throughput surgical robot</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>npj Vaccines (May 2026) identifies an LNP-mRNA formulation with improved immunogenicity-reactogenicity profile; IL-1 is implicated in adverse reactions but dispensable for humoral immunity.</t>
+          <t>Neuralink (May 7, 2026) outlined plans for high-volume BCI production paired with a streamlined, largely automated implantation procedure, with the robot accessing arbitrary cortical targets via threads through the dura.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41541-026-01441-9</t>
+          <t>https://x.com/elonmusk/status/2006513491105165411 | https://yourstory.com/2026/05/neuralink-surgical-robot-brain-interface-2026</t>
         </is>
       </c>
     </row>
@@ -12060,17 +12040,17 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>OspA mRNA-LNP vaccine elicits borreliacidal antibodies in mice</t>
+          <t>Reduced-reactogenicity LNP-mRNA design preserves antibody response</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>npj Vaccines (May 2026) reports an OspA-encoding nucleoside-modified mRNA-LNP vaccine driving complement-dependent spirochete killing in mouse models, extending mRNA vaccine applications to Lyme disease.</t>
+          <t>npj Vaccines (May 2026) identifies an LNP-mRNA formulation with improved immunogenicity-reactogenicity profile; IL-1 is implicated in adverse reactions but dispensable for humoral immunity.</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41541-026-01451-7</t>
+          <t>https://www.nature.com/articles/s41541-026-01441-9</t>
         </is>
       </c>
     </row>
@@ -12092,27 +12072,27 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_SUB_IDEA</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>#10 Renewables + battery cost collapse</t>
+          <t>#05 mRNA vaccines + LNP delivery</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>IRENA: firm 24/7 solar+storage hits $54-82/MWh in best regions</t>
+          <t>OspA mRNA-LNP vaccine elicits borreliacidal antibodies in mice</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>IRENA's May 6 outlook puts levelized costs for firm 24/7 solar-plus-storage at $54-82/MWh in high-irradiance regions, undercutting new-build coal and gas in many markets.</t>
+          <t>npj Vaccines (May 2026) reports an OspA-encoding nucleoside-modified mRNA-LNP vaccine driving complement-dependent spirochete killing in mouse models, extending mRNA vaccine applications to Lyme disease.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>https://www.irena.org/News/pressreleases/2026/May/24-7-Renewables-Outcompete-Fossil-Fuels-on-Firm-Costs | https://www.pv-magazine.com/2026/05/06/firm-solar-and-storage-costs-fall-to-54-mwh-says-irena/</t>
+          <t>https://www.nature.com/articles/s41541-026-01451-7</t>
         </is>
       </c>
     </row>
@@ -12139,22 +12119,22 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>#08 Quantum error correction (logical qubits below threshold)</t>
+          <t>#10 Renewables + battery cost collapse</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>QuEra-Harvard-MIT demonstrate 2:1 physical-to-logical qubit ratio</t>
+          <t>IRENA: firm 24/7 solar+storage hits $54-82/MWh in best regions</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>QuEra, Harvard, and MIT reported logical-qubit memory built from just 2 physical qubits with per-round error rates around 1.3e-13, far below typical &gt;10:1 prior overheads.</t>
+          <t>IRENA's May 6 outlook puts levelized costs for firm 24/7 solar-plus-storage at $54-82/MWh in high-irradiance regions, undercutting new-build coal and gas in many markets.</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>https://www.mariakorolov.com/2026/quera-claims-quantum-error-correction-breakthrough-with-2-to-1-qubit-ratio/ | https://quantumcomputingreport.com/quera-harvard-and-mit-demonstrate-21-physical-to-logical-qubit-ratio/</t>
+          <t>https://www.irena.org/News/pressreleases/2026/May/24-7-Renewables-Outcompete-Fossil-Fuels-on-Firm-Costs | https://www.pv-magazine.com/2026/05/06/firm-solar-and-storage-costs-fall-to-54-mwh-says-irena/</t>
         </is>
       </c>
     </row>
@@ -12176,7 +12156,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -12186,17 +12166,17 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Ising: open AI models for QEC decoding and calibration</t>
+          <t>QuEra-Harvard-MIT demonstrate 2:1 physical-to-logical qubit ratio</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA released the open-source Ising family (35B Calibration VLM + Decoding CNN) reporting ~2.5x speedup and ~3x accuracy improvement vs classical decoders, with sub-microsecond error-correction latency.</t>
+          <t>QuEra, Harvard, and MIT reported logical-qubit memory built from just 2 physical qubits with per-round error rates around 1.3e-13, far below typical &gt;10:1 prior overheads.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/nvidia-launches-ising-the-worlds-first-open-ai-models-to-accelerate-the-path-to-useful-quantum-computers | https://developer.nvidia.com/blog/nvidia-ising-introduces-ai-powered-workflows-to-build-fault-tolerant-quantum-systems/</t>
+          <t>https://www.mariakorolov.com/2026/quera-claims-quantum-error-correction-breakthrough-with-2-to-1-qubit-ratio/ | https://quantumcomputingreport.com/quera-harvard-and-mit-demonstrate-21-physical-to-logical-qubit-ratio/</t>
         </is>
       </c>
     </row>
@@ -12218,27 +12198,27 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>UPDATED_FACT</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>#09 Reusable rockets (Falcon 9 + Starship catch)</t>
+          <t>#08 Quantum error correction (logical qubits below threshold)</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Falcon 9 deploys CAS500-2 plus 44 rideshare payloads</t>
+          <t>NVIDIA Ising: open AI models for QEC decoding and calibration</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>SpaceX flew a Falcon 9 from Vandenberg on May 2-3 deploying South Korea's CAS500-2 Earth-observation satellite plus 44 additional payloads, continuing a high-cadence rideshare cadence.</t>
+          <t>NVIDIA released the open-source Ising family (35B Calibration VLM + Decoding CNN) reporting ~2.5x speedup and ~3x accuracy improvement vs classical decoders, with sub-microsecond error-correction latency.</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>https://spaceflightnow.com/2026/05/02/live-coverage-spacex-to-launch-south-korean-earth-observation-satellite-44-more-payloads-on-overnight-falcon-9-rideshare-mission/ | https://www.space.com/space-exploration/launches-spacecraft/spacex-falcon-9-launch-cas500-2-mission-45-satellites</t>
+          <t>https://nvidianews.nvidia.com/news/nvidia-launches-ising-the-worlds-first-open-ai-models-to-accelerate-the-path-to-useful-quantum-computers | https://developer.nvidia.com/blog/nvidia-ising-introduces-ai-powered-workflows-to-build-fault-tolerant-quantum-systems/</t>
         </is>
       </c>
     </row>
@@ -12260,7 +12240,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>NEW_FRONTIER</t>
+          <t>UPDATED_FACT</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -12270,17 +12250,17 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Starship Flight 12 (V3) targeted mid-May from Pad 2</t>
+          <t>Falcon 9 deploys CAS500-2 plus 44 rideshare payloads</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>SpaceX is targeting May 12-18 for Starship Flight 12 with the new V3 architecture (~100+ MT to LEO), and the first launch from the newly-operational Pad 2 at Starbase.</t>
+          <t>SpaceX flew a Falcon 9 from Vandenberg on May 2-3 deploying South Korea's CAS500-2 Earth-observation satellite plus 44 additional payloads, continuing a high-cadence rideshare cadence.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>https://www.basenor.com/blogs/news/starship-flight-12-targets-mid-may-with-new-v3-vehicle | https://www.nasaspaceflight.com/2026/05/spacex-mid-may-starship-flight-12-revised-trajectory/</t>
+          <t>https://spaceflightnow.com/2026/05/02/live-coverage-spacex-to-launch-south-korean-earth-observation-satellite-44-more-payloads-on-overnight-falcon-9-rideshare-mission/ | https://www.space.com/space-exploration/launches-spacecraft/spacex-falcon-9-launch-cas500-2-mission-45-satellites</t>
         </is>
       </c>
     </row>
@@ -12292,35 +12272,39 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>BASE_RUN</t>
+          <t>WEEKLY_UPDATE</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Base set extended from 11 to 15 breakthroughs: added humanoid robotics (#12), fusion energy (#13), brain-computer interfaces (#14), AI accelerators / advanced compute (#15). Two new domains introduced (ROBOTICS, HARDWARE).</t>
+          <t>Quietly busy week dominated by AI-tooling, quantum, and clinical-bio progress. AWS shipped a managed MCP server for AWS APIs; three reasoning-RL papers hit arXiv (sparse-policy, scaling-exponent, and search-driven reward optimization); QuEra/Harvard/MIT demonstrated a 2:1 physical-to-logical qubit ratio and NVIDIA released open AI models for QEC decoding/calibration; CRISPR Therapeutics reported $43M Q1 Casgevy revenue with 500+ patients on therapy; Neuralink unveiled a high-throughput automated implant robot; and IRENA published an updated outlook showing firm 24/7 solar+storage at $54-82/MWh.</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>NEW_BREAKTHROUGH</t>
+          <t>NEW_FRONTIER</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>#12 Humanoid robotics</t>
+          <t>#09 Reusable rockets (Falcon 9 + Starship catch)</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Added breakthrough: Humanoid robotics</t>
+          <t>Starship Flight 12 (V3) targeted mid-May from Pad 2</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Humanoid robotics moved from research demos to low-volume industrial production between late 2024 and May 2026 — Tesla and Boston Dynamics in factories, Figure on the BMW line, 1X taking consumer pre-orders, with VLA models (RT-2, π0, Helix) finally enabling task generalization beyond hand-coded behaviors.</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr"/>
+          <t>SpaceX is targeting May 12-18 for Starship Flight 12 with the new V3 architecture (~100+ MT to LEO), and the first launch from the newly-operational Pad 2 at Starbase.</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.basenor.com/blogs/news/starship-flight-12-targets-mid-may-with-new-v3-vehicle | https://www.nasaspaceflight.com/2026/05/spacex-mid-may-starship-flight-12-revised-trajectory/</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -12345,17 +12329,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>#13 Fusion energy</t>
+          <t>#12 Humanoid robotics</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Added breakthrough: Fusion energy</t>
+          <t>Added breakthrough: Humanoid robotics</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Fusion went from public-science promise to active commercial track between 2022 and 2026: NIF demonstrated repeatable net energy gain, CFS broke ground on SPARC with HTS magnets, and Helion shipped a D-T plasma machine on the way to a 50 MW commercial PPA with Microsoft.</t>
+          <t>Humanoid robotics moved from research demos to low-volume industrial production between late 2024 and May 2026 — Tesla and Boston Dynamics in factories, Figure on the BMW line, 1X taking consumer pre-orders, with VLA models (RT-2, π0, Helix) finally enabling task generalization beyond hand-coded behaviors.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -12383,17 +12367,17 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>#14 Brain-computer interfaces</t>
+          <t>#13 Fusion energy</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Added breakthrough: Brain-computer interfaces</t>
+          <t>Added breakthrough: Fusion energy</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>BCIs crossed from lab to early commercial reality between 2024 and 2026: Neuralink put 5+ patients on the Telepathy implant, Precision Neuroscience took home the first wireless-cortical-BCI 510(k), BrainGate hit 110 cpm bimanual typing, UCSF restored speech at 78 wpm, and Meta shipped a 20.9 wpm sEMG wristband to consumers.</t>
+          <t>Fusion went from public-science promise to active commercial track between 2022 and 2026: NIF demonstrated repeatable net energy gain, CFS broke ground on SPARC with HTS magnets, and Helion shipped a D-T plasma machine on the way to a 50 MW commercial PPA with Microsoft.</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr"/>
@@ -12421,17 +12405,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>#15 AI accelerators / advanced compute</t>
+          <t>#14 Brain-computer interfaces</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Added breakthrough: AI accelerators / advanced compute</t>
+          <t>Added breakthrough: Brain-computer interfaces</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>GPU-dominated AI compute fractured into specialized lanes between 2024 and 2026 — wafer-scale (Cerebras), inference ASICs (Groq, Etched), photonic interconnect (Lightmatter), and per-hyperscaler custom silicon (TPU/Trainium/Maia/MTIA) — pulling 20–70% of opex out of training and inference.</t>
+          <t>BCIs crossed from lab to early commercial reality between 2024 and 2026: Neuralink put 5+ patients on the Telepathy implant, Precision Neuroscience took home the first wireless-cortical-BCI 510(k), BrainGate hit 110 cpm bimanual typing, UCSF restored speech at 78 wpm, and Meta shipped a 20.9 wpm sEMG wristband to consumers.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -12449,26 +12433,64 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
+          <t>Base set extended from 11 to 15 breakthroughs: added humanoid robotics (#12), fusion energy (#13), brain-computer interfaces (#14), AI accelerators / advanced compute (#15). Two new domains introduced (ROBOTICS, HARDWARE).</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>NEW_BREAKTHROUGH</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>#15 AI accelerators / advanced compute</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Added breakthrough: AI accelerators / advanced compute</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>GPU-dominated AI compute fractured into specialized lanes between 2024 and 2026 — wafer-scale (Cerebras), inference ASICs (Groq, Etched), photonic interconnect (Lightmatter), and per-hyperscaler custom silicon (TPU/Trainium/Maia/MTIA) — pulling 20–70% of opex out of training and inference.</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>BASE_RUN</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
           <t>Initial base-truth capture across 11 breakthroughs: 62 named people, 56 sub-ideas, 55 frontier bullets, 39 watch-list picks, 150 unique source URLs.</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>BASE</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>All 11 breakthroughs captured (10 from spec + self-driving as #11)</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>Transformers/LLMs, RLHF/reasoning, diffusion, AlphaFold, mRNA, GLP-1, CRISPR, QEC, reusable rockets, batteries, plus self-driving cars/robotaxis. MCP added as a sub-idea under transformers, agentic AI under reasoning.</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>